<commit_message>
chore(pims): pre-existing tree changes (Slice 3 field-flow + photo embed)
Pre-staged changes that predate the precedent-import work, separated from
slice-1 to keep per-slice history clean:
- recommendation added to STAGING_COPY_FIELDS with field-semantics comment
  (polished narrative vs short action-register entry)
- audit report renderer pre-fetches photos for ALL observations, not just
  open actions, so checklist rows can also show inline thumbnails
- audit_report_docx.py adjustments
- audit_checklist.xlsx update
- removed unused RPD_SSA_template.docx and audit_report_template.docx

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pims/audit_checklist.xlsx
+++ b/pims/audit_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlanRichardson\gatekeeper\pims\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{810251A2-55FA-4248-B8C6-FC3136757945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386F8446-28E9-425A-B002-422A16D7CE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30405" yWindow="-2970" windowWidth="21690" windowHeight="14235" activeTab="1" xr2:uid="{91678ABD-00CB-4CA9-BCA2-78B54436A12B}"/>
+    <workbookView xWindow="8760" yWindow="1032" windowWidth="14376" windowHeight="12180" activeTab="1" xr2:uid="{91678ABD-00CB-4CA9-BCA2-78B54436A12B}"/>
   </bookViews>
   <sheets>
     <sheet name="&lt;$250K_inspection_checklist" sheetId="2" r:id="rId1"/>
@@ -2591,7 +2591,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>194</v>
       </c>
@@ -2602,7 +2602,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>194</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>194</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>194</v>
       </c>
@@ -2646,7 +2646,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>194</v>
       </c>
@@ -2657,7 +2657,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>194</v>
       </c>
@@ -2712,7 +2712,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>194</v>
       </c>
@@ -2734,7 +2734,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>194</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>194</v>
       </c>

</xml_diff>